<commit_message>
data: se termina de anonimizar los .xlsx de muestra y se agrega la jornada 07-09
- Se vacía también la columna de correo en los seis exports de Momento 4 y en
  Participacion2026-31-08-all.xlsx. Junto con el vaciado previo de nombres,
  cédula y código de estudiante, estos archivos ya no llevan ningún dato
  personal; siguen sirviendo como muestra del formato (encabezados y demás
  columnas intactos).
- Se versiona Participacion2026-07-09.xlsx (320 filas, jornada de Girardot) con
  las mismas columnas PII vaciadas. Sus datos ya están en Postgres.

Ninguno de estos .xlsx lo lee la app —los módulos de /admin viven en
Postgres—, así que el cambio no toca código ni cifras de los paneles.
</commit_message>
<xml_diff>
--- a/data/source-momento4-planeacion-territorial/Experiencia_ _Transformaciones que nos conectan_. (UC INTELIGENTE)(1-53).xlsx
+++ b/data/source-momento4-planeacion-territorial/Experiencia_ _Transformaciones que nos conectan_. (UC INTELIGENTE)(1-53).xlsx
@@ -124,10 +124,10 @@
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
-        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
-        <a:font script="Hans" typeface="å®ä½"/>
-        <a:font script="Hant" typeface="æ°ç´°æé«"/>
+        <a:font script="Jpan" typeface="Ã¯Â¼Â­Ã¯Â¼Â³ Ã¯Â¼Â°Ã£ÂÂ´Ã£ÂÂ·Ã£ÂÂÃ£ÂÂ¯"/>
+        <a:font script="Hang" typeface="Ã«Â§ÂÃ¬ÂÂ ÃªÂ³Â Ã«ÂÂ"/>
+        <a:font script="Hans" typeface="Ã¥Â®ÂÃ¤Â½Â"/>
+        <a:font script="Hant" typeface="Ã¦ÂÂ°Ã§Â´Â°Ã¦ÂÂÃ©Â«Â"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -176,10 +176,10 @@
         <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
-        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
-        <a:font script="Hans" typeface="å®ä½"/>
-        <a:font script="Hant" typeface="æ°ç´°æé«"/>
+        <a:font script="Jpan" typeface="Ã¯Â¼Â­Ã¯Â¼Â³ Ã¯Â¼Â°Ã£ÂÂ´Ã£ÂÂ·Ã£ÂÂÃ£ÂÂ¯"/>
+        <a:font script="Hang" typeface="Ã«Â§ÂÃ¬ÂÂ ÃªÂ³Â Ã«ÂÂ"/>
+        <a:font script="Hans" typeface="Ã¥Â®ÂÃ¤Â½Â"/>
+        <a:font script="Hant" typeface="Ã¦ÂÂ°Ã§Â´Â°Ã¦ÂÂÃ©Â«Â"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -496,7 +496,7 @@
         <v>46252.40724537037</v>
       </c>
       <c r="D2" t="str">
-        <v>nestorjgarcia@ucundinamarca.edu.co</v>
+        <v/>
       </c>
       <c r="E2" t="str">
         <v/>
@@ -525,7 +525,7 @@
         <v>46252.40806712963</v>
       </c>
       <c r="D3" t="str">
-        <v>iovelasquez@ucundinamarca.edu.co</v>
+        <v/>
       </c>
       <c r="E3" t="str">
         <v/>
@@ -554,7 +554,7 @@
         <v>46252.41583333333</v>
       </c>
       <c r="D4" t="str">
-        <v>dfpachon@ucundinamarca.edu.co</v>
+        <v/>
       </c>
       <c r="E4" t="str">
         <v/>
@@ -583,7 +583,7 @@
         <v>46252.41646990741</v>
       </c>
       <c r="D5" t="str">
-        <v>sfvergara@ucundinamarca.edu.co</v>
+        <v/>
       </c>
       <c r="E5" t="str">
         <v/>
@@ -615,7 +615,7 @@
         <v>46252.41677083333</v>
       </c>
       <c r="D6" t="str">
-        <v>cbosa@ucundinamarca.edu.co</v>
+        <v/>
       </c>
       <c r="E6" t="str">
         <v/>
@@ -647,7 +647,7 @@
         <v>46252.41679398148</v>
       </c>
       <c r="D7" t="str">
-        <v>smurciac@ucundinamarca.edu.co</v>
+        <v/>
       </c>
       <c r="E7" t="str">
         <v/>
@@ -679,7 +679,7 @@
         <v>46252.422789351855</v>
       </c>
       <c r="D8" t="str">
-        <v>rmunevar@ucundinamarca.edu.co</v>
+        <v/>
       </c>
       <c r="E8" t="str">
         <v/>
@@ -705,7 +705,7 @@
         <v>46252.42412037037</v>
       </c>
       <c r="D9" t="str">
-        <v>clorenarodriguez@ucundinamarca.edu.co</v>
+        <v/>
       </c>
       <c r="E9" t="str">
         <v/>
@@ -737,7 +737,7 @@
         <v>46252.43157407407</v>
       </c>
       <c r="D10" t="str">
-        <v>vnancy@ucundinamarca.edu.co</v>
+        <v/>
       </c>
       <c r="E10" t="str">
         <v/>
@@ -769,7 +769,7 @@
         <v>46252.44027777778</v>
       </c>
       <c r="D11" t="str">
-        <v>ncrubio@ucundinamarca.edu.co</v>
+        <v/>
       </c>
       <c r="E11" t="str">
         <v/>
@@ -801,7 +801,7 @@
         <v>46252.64637731481</v>
       </c>
       <c r="D12" t="str">
-        <v>afcarrilloavila@ucundinamarca.edu.co</v>
+        <v/>
       </c>
       <c r="E12" t="str">
         <v/>
@@ -830,7 +830,7 @@
         <v>46252.64655092593</v>
       </c>
       <c r="D13" t="str">
-        <v>sbravog@ucundinamarca.edu.co</v>
+        <v/>
       </c>
       <c r="E13" t="str">
         <v/>
@@ -859,7 +859,7 @@
         <v>46252.64670138889</v>
       </c>
       <c r="D14" t="str">
-        <v>atota@ucundinamarca.edu.co</v>
+        <v/>
       </c>
       <c r="E14" t="str">
         <v/>
@@ -885,7 +885,7 @@
         <v>46252.64797453704</v>
       </c>
       <c r="D15" t="str">
-        <v>yessicatrodriguez@ucundinamarca.edu.co</v>
+        <v/>
       </c>
       <c r="E15" t="str">
         <v/>
@@ -914,7 +914,7 @@
         <v>46252.647997685184</v>
       </c>
       <c r="D16" t="str">
-        <v>angiecrojas@ucundinamarca.edu.co</v>
+        <v/>
       </c>
       <c r="E16" t="str">
         <v/>
@@ -943,7 +943,7 @@
         <v>46252.64842592592</v>
       </c>
       <c r="D17" t="str">
-        <v>nlcruz@ucundinamarca.edu.co</v>
+        <v/>
       </c>
       <c r="E17" t="str">
         <v/>
@@ -972,7 +972,7 @@
         <v>46252.648506944446</v>
       </c>
       <c r="D18" t="str">
-        <v>nleonr@ucundinamarca.edu.co</v>
+        <v/>
       </c>
       <c r="E18" t="str">
         <v/>
@@ -1001,7 +1001,7 @@
         <v>46252.64921296296</v>
       </c>
       <c r="D19" t="str">
-        <v>lncajamarca@ucundinamarca.edu.co</v>
+        <v/>
       </c>
       <c r="E19" t="str">
         <v/>
@@ -1033,7 +1033,7 @@
         <v>46252.65453703704</v>
       </c>
       <c r="D20" t="str">
-        <v>empachon@ucundinamarca.edu.co</v>
+        <v/>
       </c>
       <c r="E20" t="str">
         <v/>
@@ -1062,7 +1062,7 @@
         <v>46252.65493055555</v>
       </c>
       <c r="D21" t="str">
-        <v>hacorredor@ucundinamarca.edu.co</v>
+        <v/>
       </c>
       <c r="E21" t="str">
         <v/>
@@ -1091,7 +1091,7 @@
         <v>46252.65578703704</v>
       </c>
       <c r="D22" t="str">
-        <v>jcarinagomez@ucundinamarca.edu.co</v>
+        <v/>
       </c>
       <c r="E22" t="str">
         <v/>
@@ -1117,7 +1117,7 @@
         <v>46252.65660879629</v>
       </c>
       <c r="D23" t="str">
-        <v>hcarolinasierra@ucundinamarca.edu.co</v>
+        <v/>
       </c>
       <c r="E23" t="str">
         <v/>
@@ -1149,7 +1149,7 @@
         <v>46252.657118055555</v>
       </c>
       <c r="D24" t="str">
-        <v>yzsantana@ucundinamarca.edu.co</v>
+        <v/>
       </c>
       <c r="E24" t="str">
         <v/>
@@ -1181,7 +1181,7 @@
         <v>46252.65752314815</v>
       </c>
       <c r="D25" t="str">
-        <v>vjcastro@ucundinamarca.edu.co</v>
+        <v/>
       </c>
       <c r="E25" t="str">
         <v/>
@@ -1213,7 +1213,7 @@
         <v>46252.66488425926</v>
       </c>
       <c r="D26" t="str">
-        <v>dsantiagocasallas@ucundinamarca.edu.co</v>
+        <v/>
       </c>
       <c r="E26" t="str">
         <v/>
@@ -1242,7 +1242,7 @@
         <v>46252.665243055555</v>
       </c>
       <c r="D27" t="str">
-        <v>paulaaperez@ucundinamarca.edu.co</v>
+        <v/>
       </c>
       <c r="E27" t="str">
         <v/>
@@ -1268,7 +1268,7 @@
         <v>46252.66546296296</v>
       </c>
       <c r="D28" t="str">
-        <v>kxvillamil@ucundinamarca.edu.co</v>
+        <v/>
       </c>
       <c r="E28" t="str">
         <v/>
@@ -1300,7 +1300,7 @@
         <v>46252.66587962963</v>
       </c>
       <c r="D29" t="str">
-        <v>krociomurcia@ucundinamarca.edu.co</v>
+        <v/>
       </c>
       <c r="E29" t="str">
         <v/>
@@ -1332,7 +1332,7 @@
         <v>46252.666875</v>
       </c>
       <c r="D30" t="str">
-        <v>mehueso@ucundinamarca.edu.co</v>
+        <v/>
       </c>
       <c r="E30" t="str">
         <v/>
@@ -1364,7 +1364,7 @@
         <v>46252.666921296295</v>
       </c>
       <c r="D31" t="str">
-        <v>ynmolina@ucundinamarca.edu.co</v>
+        <v/>
       </c>
       <c r="E31" t="str">
         <v/>
@@ -1396,7 +1396,7 @@
         <v>46252.66787037037</v>
       </c>
       <c r="D32" t="str">
-        <v>jbriseno@ucundinamarca.edu.co</v>
+        <v/>
       </c>
       <c r="E32" t="str">
         <v/>
@@ -1428,7 +1428,7 @@
         <v>46252.67240740741</v>
       </c>
       <c r="D33" t="str">
-        <v>eestibengarzon@ucundinamarca.edu.co</v>
+        <v/>
       </c>
       <c r="E33" t="str">
         <v/>
@@ -1457,7 +1457,7 @@
         <v>46252.67261574074</v>
       </c>
       <c r="D34" t="str">
-        <v>ahvanegas@ucundinamarca.edu.co</v>
+        <v/>
       </c>
       <c r="E34" t="str">
         <v/>
@@ -1486,7 +1486,7 @@
         <v>46252.673101851855</v>
       </c>
       <c r="D35" t="str">
-        <v>karendortiz@ucundinamarca.edu.co</v>
+        <v/>
       </c>
       <c r="E35" t="str">
         <v/>
@@ -1518,7 +1518,7 @@
         <v>46252.67340277778</v>
       </c>
       <c r="D36" t="str">
-        <v>nmhuertas@ucundinamarca.edu.co</v>
+        <v/>
       </c>
       <c r="E36" t="str">
         <v/>
@@ -1550,7 +1550,7 @@
         <v>46252.67364583333</v>
       </c>
       <c r="D37" t="str">
-        <v>ndalarcon@ucundinamarca.edu.co</v>
+        <v/>
       </c>
       <c r="E37" t="str">
         <v/>
@@ -1579,7 +1579,7 @@
         <v>46252.67380787037</v>
       </c>
       <c r="D38" t="str">
-        <v>jpaolamontanez@ucundinamarca.edu.co</v>
+        <v/>
       </c>
       <c r="E38" t="str">
         <v/>
@@ -1608,7 +1608,7 @@
         <v>46252.677407407406</v>
       </c>
       <c r="D39" t="str">
-        <v>jefersonalejandroramirez@ucundinamarca.edu.co</v>
+        <v/>
       </c>
       <c r="E39" t="str">
         <v/>
@@ -1637,7 +1637,7 @@
         <v>46252.67763888889</v>
       </c>
       <c r="D40" t="str">
-        <v>rguilombo@ucundinamarca.edu.co</v>
+        <v/>
       </c>
       <c r="E40" t="str">
         <v/>
@@ -1666,7 +1666,7 @@
         <v>46252.67899305555</v>
       </c>
       <c r="D41" t="str">
-        <v>yandreyrincon@ucundinamarca.edu.co</v>
+        <v/>
       </c>
       <c r="E41" t="str">
         <v/>
@@ -1695,7 +1695,7 @@
         <v>46252.683125</v>
       </c>
       <c r="D42" t="str">
-        <v>lvchiquiza@ucundinamarca.edu.co</v>
+        <v/>
       </c>
       <c r="E42" t="str">
         <v/>
@@ -1724,7 +1724,7 @@
         <v>46252.68347222222</v>
       </c>
       <c r="D43" t="str">
-        <v>nalavardo@ucundinamarca.edu.co</v>
+        <v/>
       </c>
       <c r="E43" t="str">
         <v/>
@@ -1756,7 +1756,7 @@
         <v>46252.806805555556</v>
       </c>
       <c r="D44" t="str">
-        <v>ybeltran@ucundinamarca.edu.co</v>
+        <v/>
       </c>
       <c r="E44" t="str">
         <v/>
@@ -1788,7 +1788,7 @@
         <v>46252.80725694444</v>
       </c>
       <c r="D45" t="str">
-        <v>ylrobayo@ucundinamarca.edu.co</v>
+        <v/>
       </c>
       <c r="E45" t="str">
         <v/>
@@ -1820,7 +1820,7 @@
         <v>46252.80784722222</v>
       </c>
       <c r="D46" t="str">
-        <v>nfarfan@ucundinamarca.edu.co</v>
+        <v/>
       </c>
       <c r="E46" t="str">
         <v/>
@@ -1852,7 +1852,7 @@
         <v>46252.812569444446</v>
       </c>
       <c r="D47" t="str">
-        <v>erpena@ucundinamarca.edu.co</v>
+        <v/>
       </c>
       <c r="E47" t="str">
         <v/>
@@ -1884,7 +1884,7 @@
         <v>46252.81348379629</v>
       </c>
       <c r="D48" t="str">
-        <v>jpaolacastiblanco@ucundinamarca.edu.co</v>
+        <v/>
       </c>
       <c r="E48" t="str">
         <v/>
@@ -1919,7 +1919,7 @@
         <v>46252.82413194444</v>
       </c>
       <c r="D49" t="str">
-        <v>anonymous</v>
+        <v/>
       </c>
       <c r="I49" t="str">
         <v>Creadores de Oportunidades (estudiantes)</v>
@@ -1951,7 +1951,7 @@
         <v>46252.82506944444</v>
       </c>
       <c r="D50" t="str">
-        <v>anonymous</v>
+        <v/>
       </c>
       <c r="I50" t="str">
         <v>Graduados</v>
@@ -1983,7 +1983,7 @@
         <v>46252.83712962963</v>
       </c>
       <c r="D51" t="str">
-        <v>anonymous</v>
+        <v/>
       </c>
       <c r="I51" t="str">
         <v>Graduados</v>
@@ -2015,7 +2015,7 @@
         <v>46252.83738425926</v>
       </c>
       <c r="D52" t="str">
-        <v>anonymous</v>
+        <v/>
       </c>
       <c r="I52" t="str">
         <v>Graduados</v>
@@ -2047,7 +2047,7 @@
         <v>46252.83765046296</v>
       </c>
       <c r="D53" t="str">
-        <v>anonymous</v>
+        <v/>
       </c>
       <c r="I53" t="str">
         <v>Graduados</v>
@@ -2079,7 +2079,7 @@
         <v>46252.842361111114</v>
       </c>
       <c r="D54" t="str">
-        <v>anonymous</v>
+        <v/>
       </c>
       <c r="I54" t="str">
         <v>Graduados</v>

</xml_diff>